<commit_message>
docs: record team decisions as assumptions, set license holder and AI-002 verifier [Deliverables 14, 18]
- README Assumptions and RTM 'Organizer Questions' hold the 7 team decisions
- T-01..T-13 back to In Progress until working code uses each technology

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentation/SupportNova_RTM.xlsx
+++ b/documentation/SupportNova_RTM.xlsx
@@ -18982,12 +18982,12 @@
       </c>
       <c r="O261" s="32" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="P261" s="32" t="inlineStr">
         <is>
-          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; libraries pinned in requirements.txt (implementation evidence added by later slices)</t>
+          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; library pinned in requirements.txt. Moves to Done when a slice uses it in working code.</t>
         </is>
       </c>
     </row>
@@ -19052,12 +19052,12 @@
       </c>
       <c r="O262" s="32" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="P262" s="32" t="inlineStr">
         <is>
-          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; libraries pinned in requirements.txt (implementation evidence added by later slices)</t>
+          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; library pinned in requirements.txt. Moves to Done when a slice uses it in working code.</t>
         </is>
       </c>
     </row>
@@ -19122,12 +19122,12 @@
       </c>
       <c r="O263" s="32" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="P263" s="32" t="inlineStr">
         <is>
-          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; libraries pinned in requirements.txt (implementation evidence added by later slices)</t>
+          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; library pinned in requirements.txt. Moves to Done when a slice uses it in working code.</t>
         </is>
       </c>
     </row>
@@ -19192,12 +19192,12 @@
       </c>
       <c r="O264" s="32" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="P264" s="32" t="inlineStr">
         <is>
-          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; libraries pinned in requirements.txt (implementation evidence added by later slices)</t>
+          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; library pinned in requirements.txt. Moves to Done when a slice uses it in working code.</t>
         </is>
       </c>
     </row>
@@ -19262,12 +19262,12 @@
       </c>
       <c r="O265" s="32" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="P265" s="32" t="inlineStr">
         <is>
-          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; libraries pinned in requirements.txt (implementation evidence added by later slices)</t>
+          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; library pinned in requirements.txt. Moves to Done when a slice uses it in working code.</t>
         </is>
       </c>
     </row>
@@ -19332,12 +19332,12 @@
       </c>
       <c r="O266" s="32" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="P266" s="32" t="inlineStr">
         <is>
-          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; libraries pinned in requirements.txt (implementation evidence added by later slices)</t>
+          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; library pinned in requirements.txt. Moves to Done when a slice uses it in working code.</t>
         </is>
       </c>
     </row>
@@ -19402,12 +19402,12 @@
       </c>
       <c r="O267" s="32" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="P267" s="32" t="inlineStr">
         <is>
-          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; libraries pinned in requirements.txt (implementation evidence added by later slices)</t>
+          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; library pinned in requirements.txt. Moves to Done when a slice uses it in working code.</t>
         </is>
       </c>
     </row>
@@ -19472,12 +19472,12 @@
       </c>
       <c r="O268" s="32" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="P268" s="32" t="inlineStr">
         <is>
-          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; libraries pinned in requirements.txt (implementation evidence added by later slices)</t>
+          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; library pinned in requirements.txt. Moves to Done when a slice uses it in working code.</t>
         </is>
       </c>
     </row>
@@ -19542,12 +19542,12 @@
       </c>
       <c r="O269" s="32" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="P269" s="32" t="inlineStr">
         <is>
-          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; libraries pinned in requirements.txt (implementation evidence added by later slices)</t>
+          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; library pinned in requirements.txt. Moves to Done when a slice uses it in working code.</t>
         </is>
       </c>
     </row>
@@ -19612,12 +19612,12 @@
       </c>
       <c r="O270" s="32" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="P270" s="32" t="inlineStr">
         <is>
-          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; libraries pinned in requirements.txt (implementation evidence added by later slices)</t>
+          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; library pinned in requirements.txt. Moves to Done when a slice uses it in working code.</t>
         </is>
       </c>
     </row>
@@ -19682,12 +19682,12 @@
       </c>
       <c r="O271" s="32" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="P271" s="32" t="inlineStr">
         <is>
-          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; libraries pinned in requirements.txt (implementation evidence added by later slices)</t>
+          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; library pinned in requirements.txt. Moves to Done when a slice uses it in working code.</t>
         </is>
       </c>
     </row>
@@ -19752,12 +19752,12 @@
       </c>
       <c r="O272" s="32" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="P272" s="32" t="inlineStr">
         <is>
-          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; libraries pinned in requirements.txt (implementation evidence added by later slices)</t>
+          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; library pinned in requirements.txt. Moves to Done when a slice uses it in working code.</t>
         </is>
       </c>
     </row>
@@ -19822,12 +19822,12 @@
       </c>
       <c r="O273" s="32" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="P273" s="32" t="inlineStr">
         <is>
-          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; libraries pinned in requirements.txt (implementation evidence added by later slices)</t>
+          <t>P01-S1: choice documented in ADR-001 and README 'Technology stack'; library pinned in requirements.txt. Moves to Done when a slice uses it in working code.</t>
         </is>
       </c>
     </row>
@@ -41899,8 +41899,16 @@
           <t>HD-06/07, CI-05, CI-14</t>
         </is>
       </c>
-      <c r="E2" s="32" t="n"/>
-      <c r="F2" s="32" t="n"/>
+      <c r="E2" s="32" t="inlineStr">
+        <is>
+          <t>Team decision (organizers not contacted): Rule matrix and all configuration are managed from the Admin UI (add/edit/delete/import); no code changes for hidden data.</t>
+        </is>
+      </c>
+      <c r="F2" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="23.85" customHeight="1" s="17">
       <c r="A3" s="31" t="n">
@@ -41921,8 +41929,16 @@
           <t>P2-01, T-08, CI-18</t>
         </is>
       </c>
-      <c r="E3" s="32" t="n"/>
-      <c r="F3" s="32" t="n"/>
+      <c r="E3" s="32" t="inlineStr">
+        <is>
+          <t>Team decision (organizers not contacted): Pipeline 2 is rules-only. No ML model of any kind.</t>
+        </is>
+      </c>
+      <c r="F3" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="23.85" customHeight="1" s="17">
       <c r="A4" s="31" t="n">
@@ -41943,8 +41959,16 @@
           <t>CI-03, D-08</t>
         </is>
       </c>
-      <c r="E4" s="32" t="n"/>
-      <c r="F4" s="32" t="n"/>
+      <c r="E4" s="32" t="inlineStr">
+        <is>
+          <t>Team decision (organizers not contacted): Unknown hidden format, so batch import supports CSV, TSV, XLSX, JSON and JSONL with column mapping.</t>
+        </is>
+      </c>
+      <c r="F4" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="23.85" customHeight="1" s="17">
       <c r="A5" s="31" t="n">
@@ -41965,8 +41989,16 @@
           <t>CI-16, D-14</t>
         </is>
       </c>
-      <c r="E5" s="32" t="n"/>
-      <c r="F5" s="32" t="n"/>
+      <c r="E5" s="32" t="inlineStr">
+        <is>
+          <t>Team decision (organizers not contacted): Design and planning within the five days is allowed.</t>
+        </is>
+      </c>
+      <c r="F5" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="23.85" customHeight="1" s="17">
       <c r="A6" s="31" t="n">
@@ -41987,8 +42019,16 @@
           <t>T-09, P2-01</t>
         </is>
       </c>
-      <c r="E6" s="32" t="n"/>
-      <c r="F6" s="32" t="n"/>
+      <c r="E6" s="32" t="inlineStr">
+        <is>
+          <t>Team decision (organizers not contacted): No embeddings in Pipeline 2. Retrieval uses BM25.</t>
+        </is>
+      </c>
+      <c r="F6" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="23.85" customHeight="1" s="17">
       <c r="A7" s="31" t="n">
@@ -42009,8 +42049,16 @@
           <t>P1-01, T-05</t>
         </is>
       </c>
-      <c r="E7" s="32" t="n"/>
-      <c r="F7" s="32" t="n"/>
+      <c r="E7" s="32" t="inlineStr">
+        <is>
+          <t>Team decision (organizers not contacted): OpenAI model through the CommandCode OpenAI-compatible gateway (ADR-007). Model ID set before P01-S6.</t>
+        </is>
+      </c>
+      <c r="F7" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="17">
       <c r="A8" s="31" t="n">
@@ -42031,8 +42079,16 @@
           <t>D-19</t>
         </is>
       </c>
-      <c r="E8" s="32" t="n"/>
-      <c r="F8" s="32" t="n"/>
+      <c r="E8" s="32" t="inlineStr">
+        <is>
+          <t>Team decision (organizers not contacted): Team of 4. No required format for the contribution record; we use documentation/team_contribution.md.</t>
+        </is>
+      </c>
+      <c r="F8" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
docs(rtm): record P01-S2 evidence, AI usage entry and app_errors sink task for P01-S3 [FR lxxiv, CN-02, Deliverable 18]
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentation/SupportNova_RTM.xlsx
+++ b/documentation/SupportNova_RTM.xlsx
@@ -2870,10 +2870,14 @@
       </c>
       <c r="O21" s="32" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="P21" s="32" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="P21" s="32" t="inlineStr">
+        <is>
+          <t>P01-S2: secrets only from env (src/core/settings.py, tests/core/test_settings.py); PII masked in logs (security/pii.py, tests/core/test_logging_masking.py); commits e5f5f00, d4c9c74, 0394b44</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="23.85" customHeight="1" s="17">
       <c r="A22" s="30" t="inlineStr">
@@ -12424,10 +12428,14 @@
       </c>
       <c r="O164" s="32" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="P164" s="32" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="P164" s="32" t="inlineStr">
+        <is>
+          <t>P01-S2: domain exceptions, error refs, capture_exception, error box (src/core/errors.py, src/app/components/error_box.py; tests/core/test_error_refs.py; commit 4183d5e). API/parsing/DB error paths and app_errors persistence follow in P01-S3, P03, P06</t>
+        </is>
+      </c>
     </row>
     <row r="165" ht="15" customHeight="1" s="17">
       <c r="A165" s="30" t="inlineStr">
@@ -30686,10 +30694,14 @@
       </c>
       <c r="O427" s="32" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="P427" s="32" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="P427" s="32" t="inlineStr">
+        <is>
+          <t>P01-S2: log masking of emails/phones/card numbers proven by tests/core/test_logging_masking.py; report in P12</t>
+        </is>
+      </c>
     </row>
     <row r="428" ht="23.85" customHeight="1" s="17">
       <c r="A428" s="31" t="inlineStr">
@@ -33132,10 +33144,14 @@
       </c>
       <c r="O462" s="32" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="P462" s="32" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="P462" s="32" t="inlineStr">
+        <is>
+          <t>P01-S2: keys read only from environment, never echoed (test_startup_error_never_echoes_secret_values, test_secrets_are_hidden_in_repr)</t>
+        </is>
+      </c>
     </row>
     <row r="463" ht="23.85" customHeight="1" s="17">
       <c r="A463" s="30" t="inlineStr">
@@ -35331,7 +35347,7 @@
       </c>
       <c r="P493" s="32" t="inlineStr">
         <is>
-          <t>P01-S1: .env git-ignored; .env.example without values (test_env_example_declares_keys_without_values, test_gitignore_keeps_env_files_out_but_allows_example); pre-commit detect-private-key</t>
+          <t>P01-S1: .env git-ignored; .env.example without values (test_env_example_declares_keys_without_values, test_gitignore_keeps_env_files_out_but_allows_example); pre-commit detect-private-key; P01-S2: SecretStr settings; secrets never echoed in startup errors (tests/core/test_settings.py)</t>
         </is>
       </c>
     </row>

</xml_diff>